<commit_message>
feat: joint skills state the stored value of their effects
JoinSkillData decoded (participants, TP divisor, Pep, power, turns, four
effect slots) and its writer made exact for all 52 entries (the third
string is a battle message). 29 sentences carry the stored chance or
amount in place of the vague word; sentences live in the rules workbook.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_rules.xlsx
+++ b/mod_project/data_tables/qol_rules.xlsx
@@ -21,6 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnemyEffects" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WordingFixes" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PartySkillBounds" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JointEffects" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JointSkillSentences" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -614,6 +616,30 @@
       <c r="B15" t="inlineStr">
         <is>
           <t>Upper bound of each party skill bonus (DT2-2 wiki), in the order the sentence names them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>JointEffects</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Joint skills: how the value of an effect is written when a sentence quotes it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>JointSkillSentences</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Joint skills: the sentence of the game with the stored value of an effect in place of {eID}. A skill without a row keeps its text.</t>
         </is>
       </c>
     </row>
@@ -2291,6 +2317,923 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Effect_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Style</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Poison</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>114</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Freeze</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>115</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Paralysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>116</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sleep</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>117</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Silence</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>118</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Stun</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>119</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Instakill</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>120</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Petrification</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>122</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Slow</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>123</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Shadow Sew</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>54</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>chance</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Turn delay</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>161</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Physical attack</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>162</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Physical defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>163</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Magic defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>166</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Physical accuracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>168</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>173</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Magic attack. Named by the game table; unit by analogy with 161</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>174</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>signed_points_pct</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Crit rate. Named by the game table; unit by analogy with 31 (points)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>169</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>signed_points_pct</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>All resistances, in points (one point is 1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>66</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>signed_num</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pep UP. Named by the game table; 80 (Pep DOWN) is stored the same way</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>105</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>HP on revival, fraction of max HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>433</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Money Loss: fraction of the gold held (DT2-2 wiki: 5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>296</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Damage cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>147</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Turns a summoned attack lasts</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>93</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Hit count</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>88</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>times</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1 + value: God Punch says "2x damage" for a stored 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>89</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Game table: 2~5 Hits</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>94</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Game table: 0~4 Hits</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>95</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Game table: 1~5 Hits</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>96</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Game table: 3~5 Hits</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentence</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Catastrophe</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inflict a powerful physical attack on one enemy. Inflicts slow ({e122}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Genocide Rain</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Rain arrows down upon all enemies across {e147} turns.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Wiki: 2 volleys, each attacks every enemy twice a turn for 4 turns</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Divine Punishment!</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Deal physical damage to an enemy row. {e119} chance of instakill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Nightmare Fall</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Deal non-elemental damage to all enemies. {e116} chance of causing sleep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Powered-Up Beatdown!</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inflict one enemy with {e96} bash attacks. {e118} chance of stun.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Psychowave</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Deal non-elemental damage and lower DEF and magic defense ({e162}) for all enemies.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The original names DEF only; the data also lowers magic defense (163), as the Japanese text says</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Avatara</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Deal physical damage and {e95} defense-piercing attacks on one enemy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gjallarhorn</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Activate Circle Brave ({e161}), Circle Protect ({e162}) and Moon Curtain ({e169}) at once.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Shortened ("all at the same time") to make room</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Suppression Arrow</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Deal damage with an {e117} chance to silence/freeze. Pierces to the back row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rapid Storm</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Form up to increase speed ({e168}) and physical accuracy ({e166}) for all allies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Evolution</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Increase magic attack ({e173}) and critical rate ({e174}) for all allies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bunker Buster</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Deal damage and reduce physical attack/defense ({e161}). Pierces to the back row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Paralyzing Wind</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Inflict a wind attack against all enemies. {e115} chance of paralysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Daruma-Drop!</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Deal physical damage, with a {e54} chance to delay the target's next turn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Testament</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Deal physical damage and use Shadow Sew ({e123}) against an enemy row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Brain Burst</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Deal physical damage to one enemy. {e113} chance of poison/paralysis/sleep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Happy Banquet</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Increase Pep ({e66}) for the ally whose Pep is the lowest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hysteric Slap</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Inflict {e94} bash attacks on an enemy row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fire of Purgatory</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Attack one enemy ({e88} damage to Undead, Demons, and Apparitions).</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Same effect and value as God Punch, which says "2x damage"</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Curse Bullet</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Waste one enemy and poison the target ({e113}) with a rare gun-type weapon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Beast Blitz</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Rough up ({e93} hits) and poison ({e113}) one enemy with the power of darkness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Durchbruch</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Fire two arrows of light that pierce to the back row and may silence ({e117}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Maid Beam</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>The deadly Maid Beam pierces to the back row and begins petrifying targets ({e120}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Feuerkraft</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Immolate all enemies and absorb their HP and TP (damage cap {e296}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Gold Power</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Hurl {e433} of your wallet at one enemy for up to {e296} damage. (You won't get it back.)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>777 Fever</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Dish out paralysis ({e115}) and 7 times the user's level in damage to all enemies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Apocrypha</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Waste one enemy and lower target's phys. DEF ({e162}) with a rare gun-type weapon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Anastasia</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Summon the goddess of life to resurrect all allies (HP {e105}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Lots Of Guns</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>With three firearms in your hands, rain lead upon your enemies at random ({e93} hits).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fix: never speak from outside the game
never speak from outside the game; build check for out-of-game words

Arcane Shield's third line is now 'Activation rate: about 15%'; the
source stays in the workbook. The build stops on any modified text that
holds a word of the sheet OutOfGameWords.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_rules.xlsx
+++ b/mod_project/data_tables/qol_rules.xlsx
@@ -24,6 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JointSkillSentences" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UniqueSkillNotes" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PartySkillBounds" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OutOfGameWords" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -652,7 +653,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Unique skills: a line added under the box for a figure that only a guide gives (it says so).</t>
+          <t>Unique skills: a line added under the box for a figure the entry does not store. In the voice of the game; its origin goes in the Source column, never in the line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>OutOfGameWords</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Hard rule of the user: no text shown in the game may break the game's voice. A text the mod writes that contains one of these words (as a whole word, any case) stops the build. Where a figure comes from is recorded in these sheets, never on screen.</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2963,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Activation rate: about 15% (player guide; the game data holds no figure)</t>
+          <t>Activation rate: about 15%</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3502,6 +3515,264 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>guide</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wiki</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>game data</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>the data</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>decoded</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>not known</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>player test</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>the game</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mod</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>vanilla</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>original text</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>unconfirmed</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>not confirmed</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tbd</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>todo</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Speaks from outside the game</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: unique skill lines say what their numbers measure
unique skill lines say what their numbers measure; Arcane Shield rate
plain
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_rules.xlsx
+++ b/mod_project/data_tables/qol_rules.xlsx
@@ -25,6 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UniqueSkillNotes" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PartySkillBounds" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OutOfGameWords" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UniqueSkillLabels" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -666,6 +667,18 @@
       <c r="B19" t="inlineStr">
         <is>
           <t>Hard rule of the user: no text shown in the game may break the game's voice. A text the mod writes that contains one of these words (as a whole word, any case) stops the build. Where a figure comes from is recorded in these sheets, never on screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>UniqueSkillLabels</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Unique skills: what the numbers of the box measure, written in place of "Lv1-9". A skill without a row keeps "Lv1-9" (what its number measures is not known).</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2976,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Activation rate: about 15%</t>
+          <t>Activation rate: 15%</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3773,6 +3786,263 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Third Eye Wide</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sugar Coma</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Furious Strike</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Alter Fate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Usurper of Souls</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Overstock Clearance</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Did You Call for Me?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tranquil Song</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Forerunner</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>The sentence says it happens sometimes ("may", "occasionally") and the entry stores one rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Elbow Grease</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Weapon modifier</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>"Increase weapon modifier": the stored value is that increase</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Wreathed in Glory</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Turn delay</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>"Decrease turn delay": the stored value is that decrease</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Maximum Maid</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Maid skill effects</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>"Increased effects for all maid skills"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Arcane Shield</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Reflected</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DT2-2 wiki pages/42.html: the stored value is the share reflected (50% at Lv1, 200% with the crown)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat: rule texts checked against the data
rule texts checked against the data; one tutorial sentence corrected in
place

Lessons, tutorials, shop talk, quest ranks and 40 quest reward lines
agree with the data. The tutorial on level reset said 'over 59'; the
lesson and the guide say 59 or greater. Script packs are patched with
same-length replacements only (sheet ScriptFixes) and installed into the
game's Script folder.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_rules.xlsx
+++ b/mod_project/data_tables/qol_rules.xlsx
@@ -26,6 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PartySkillBounds" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OutOfGameWords" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UniqueSkillLabels" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ScriptFixes" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -679,6 +680,18 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>Unique skills: what the numbers of the box measure, written in place of "Lv1-9". A skill without a row keeps "Lv1-9" (what its number measures is not known).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ScriptFixes</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Lessons, tutorials and shop dialogue: a sentence that states a rule wrongly, and its correction. The replacement must have exactly as many bytes as the original (pad with a trailing space): scripts are bytecode and are never resized.</t>
         </is>
       </c>
     </row>
@@ -4201,6 +4214,85 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Pack</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Entry</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Replacement</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Teaching.pck</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CheatsTeaching_25.adv.bin</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>When level resetting, if there is a gap of over 59 between
+your former level and the level you're resetting to,
+all your stats will increase by 1.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When level resetting, if the gap is 59 or greater between
+your former level and the level you're resetting to,
+all your stats will increase by 1. </t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>The tutorial says "over 59"; the lesson (BattleTeacher_Sp03) says "59 or greater" and so does the DT2-2 wiki (pages/79.html: a drop of 59 to 68 levels gives +1). One trailing space keeps the length.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(qol): heals shown as a multiple of RES
heals shown as a multiple of RES; wider separators in the skill boxes
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_rules.xlsx
+++ b/mod_project/data_tables/qol_rules.xlsx
@@ -4669,7 +4669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4864,6 +4864,36 @@
       <c r="C12" t="inlineStr">
         <is>
           <t>Which attacks show it. summons: only the attacks a summon of the player can use (tools/summon_data.py), the screen where these texts were seen. The user chose this on 2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>skill_wide_line</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>92</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Characters a line of the skill box may reach once its separators are widened. The content of a line is still chosen for line_width (85); the screenshot of Heal of 2026-10-05 shows a line of 73 characters ending at three quarters of the box</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>skill_separator_pad</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Spaces on each side of the bar between two items of a skill box line, when the widened line stays within skill_wide_line. The user asked for air on 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -9289,7 +9319,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HP recovery</t>
+          <t>Heals RES</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>half_mult</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tools: qol and balance text
qol and balance text: one rule for the room around the separators, the
boxes worded by hand included; Wreathed in Glory and Tranquil Song say
what the program does; the catalogue of fields brought up to date
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_rules.xlsx
+++ b/mod_project/data_tables/qol_rules.xlsx
@@ -3905,7 +3905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3944,6 +3944,23 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Read in the program: a number below 100 under 15 (0x424766, docs/FORMULAS.md 12.19). The DT2-2 wiki measured about 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tranquil Song</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Enemy ATK and INT: -10% for 4 turns</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Read in the program (docs/FORMULAS.md 12.19, 0x43749f - 0x437650): on a success every unit of the other side receives an ATK debuff and an INT debuff of -0.1 (effects 41 and 43), asked for 4 turns</t>
         </is>
       </c>
     </row>
@@ -4967,12 +4984,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Turn delay</t>
+          <t>Speed added</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>"Decrease turn delay": the stored value is that decrease</t>
+          <t>Read in the program (docs/FORMULAS.md 12.19, 0x4f72a7): the value is added to the speed of the skill or spell she uses, the figure the boxes show as "Speed: 0.95x". The label "Turn delay" read it as a cut of the delay</t>
         </is>
       </c>
     </row>

</xml_diff>